<commit_message>
test of the new tests
</commit_message>
<xml_diff>
--- a/tests/test_case.xlsx
+++ b/tests/test_case.xlsx
@@ -802,7 +802,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="68">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -999,22 +999,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1088,10 +1072,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1173,7 +1153,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AO1048576"/>
-  <sheetFormatPr defaultColWidth="7.96875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="7.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.42"/>
@@ -2357,15 +2337,15 @@
       <c r="K49" s="0"/>
       <c r="L49" s="0"/>
       <c r="M49" s="48"/>
-      <c r="N49" s="49"/>
-      <c r="O49" s="49"/>
-      <c r="P49" s="50"/>
-      <c r="Q49" s="51"/>
-      <c r="R49" s="51"/>
-      <c r="S49" s="52"/>
+      <c r="N49" s="0"/>
+      <c r="O49" s="0"/>
+      <c r="P49" s="43"/>
+      <c r="Q49" s="44"/>
+      <c r="R49" s="44"/>
+      <c r="S49" s="45"/>
       <c r="AL49" s="2"/>
       <c r="AM49" s="3"/>
-      <c r="AN49" s="53"/>
+      <c r="AN49" s="49"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="42" t="s">
@@ -2385,15 +2365,15 @@
       <c r="K50" s="0"/>
       <c r="L50" s="0"/>
       <c r="M50" s="48"/>
-      <c r="N50" s="49"/>
-      <c r="O50" s="49"/>
-      <c r="P50" s="50"/>
-      <c r="Q50" s="51"/>
-      <c r="R50" s="51"/>
-      <c r="S50" s="52"/>
+      <c r="N50" s="0"/>
+      <c r="O50" s="0"/>
+      <c r="P50" s="43"/>
+      <c r="Q50" s="44"/>
+      <c r="R50" s="44"/>
+      <c r="S50" s="45"/>
       <c r="AL50" s="2"/>
       <c r="AM50" s="3"/>
-      <c r="AN50" s="53"/>
+      <c r="AN50" s="49"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="42" t="s">
@@ -2427,7 +2407,7 @@
       <c r="S51" s="45"/>
       <c r="AL51" s="2"/>
       <c r="AM51" s="3"/>
-      <c r="AN51" s="53"/>
+      <c r="AN51" s="49"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="42"/>
@@ -2459,7 +2439,7 @@
       <c r="S52" s="45"/>
       <c r="AL52" s="2"/>
       <c r="AM52" s="3"/>
-      <c r="AN52" s="53"/>
+      <c r="AN52" s="49"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="42" t="s">
@@ -2489,7 +2469,7 @@
       <c r="S53" s="45"/>
       <c r="AL53" s="2"/>
       <c r="AM53" s="3"/>
-      <c r="AN53" s="53"/>
+      <c r="AN53" s="49"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="42"/>
@@ -2517,7 +2497,7 @@
       <c r="S54" s="45"/>
       <c r="AL54" s="2"/>
       <c r="AM54" s="3"/>
-      <c r="AN54" s="53"/>
+      <c r="AN54" s="49"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="42" t="s">
@@ -2545,7 +2525,7 @@
       <c r="S55" s="45"/>
       <c r="AL55" s="2"/>
       <c r="AM55" s="3"/>
-      <c r="AN55" s="53"/>
+      <c r="AN55" s="49"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="42"/>
@@ -2571,7 +2551,7 @@
       <c r="S56" s="45"/>
       <c r="AL56" s="2"/>
       <c r="AM56" s="3"/>
-      <c r="AN56" s="53"/>
+      <c r="AN56" s="49"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="42" t="s">
@@ -2607,7 +2587,7 @@
       <c r="S57" s="45"/>
       <c r="AL57" s="2"/>
       <c r="AM57" s="3"/>
-      <c r="AN57" s="53"/>
+      <c r="AN57" s="49"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="42"/>
@@ -2699,10 +2679,10 @@
       <c r="R59" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="S59" s="54" t="s">
+      <c r="S59" s="50" t="s">
         <v>106</v>
       </c>
-      <c r="AK59" s="55"/>
+      <c r="AK59" s="51"/>
       <c r="AL59" s="2"/>
       <c r="AM59" s="3"/>
       <c r="AN59" s="3"/>
@@ -2751,19 +2731,19 @@
       <c r="O60" s="46" t="n">
         <v>0.000712</v>
       </c>
-      <c r="P60" s="56" t="n">
+      <c r="P60" s="52" t="n">
         <v>85230.1745152193</v>
       </c>
-      <c r="Q60" s="57" t="n">
+      <c r="Q60" s="53" t="n">
         <v>293.812197080664</v>
       </c>
       <c r="R60" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S60" s="54" t="s">
+      <c r="S60" s="50" t="s">
         <v>113</v>
       </c>
-      <c r="AK60" s="55"/>
+      <c r="AK60" s="51"/>
       <c r="AL60" s="2"/>
       <c r="AM60" s="3"/>
       <c r="AN60" s="3"/>
@@ -2812,16 +2792,16 @@
       <c r="O61" s="46" t="n">
         <v>0.004005</v>
       </c>
-      <c r="P61" s="56" t="n">
+      <c r="P61" s="52" t="n">
         <v>192849.651643089</v>
       </c>
-      <c r="Q61" s="57" t="n">
+      <c r="Q61" s="53" t="n">
         <v>440.926134921357</v>
       </c>
       <c r="R61" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S61" s="54" t="s">
+      <c r="S61" s="50" t="s">
         <v>113</v>
       </c>
       <c r="AL61" s="2"/>
@@ -2873,16 +2853,16 @@
       <c r="O62" s="46" t="n">
         <v>0.003669</v>
       </c>
-      <c r="P62" s="56" t="n">
+      <c r="P62" s="52" t="n">
         <v>218506.673820773</v>
       </c>
-      <c r="Q62" s="57" t="n">
+      <c r="Q62" s="53" t="n">
         <v>469.260239787158</v>
       </c>
       <c r="R62" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S62" s="54" t="s">
+      <c r="S62" s="50" t="s">
         <v>113</v>
       </c>
       <c r="AL62" s="2"/>
@@ -2934,19 +2914,19 @@
       <c r="O63" s="46" t="n">
         <v>0.004643</v>
       </c>
-      <c r="P63" s="56" t="n">
+      <c r="P63" s="52" t="n">
         <v>88455.8671007604</v>
       </c>
-      <c r="Q63" s="57" t="n">
+      <c r="Q63" s="53" t="n">
         <v>298.338188513534</v>
       </c>
       <c r="R63" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S63" s="54" t="s">
+      <c r="S63" s="50" t="s">
         <v>113</v>
       </c>
-      <c r="AK63" s="55"/>
+      <c r="AK63" s="51"/>
       <c r="AL63" s="2"/>
       <c r="AM63" s="3"/>
       <c r="AN63" s="3"/>
@@ -2996,19 +2976,19 @@
       <c r="O64" s="46" t="n">
         <v>0.003892</v>
       </c>
-      <c r="P64" s="56" t="n">
+      <c r="P64" s="52" t="n">
         <v>169156.955820423</v>
       </c>
-      <c r="Q64" s="57" t="n">
+      <c r="Q64" s="53" t="n">
         <v>412.873655038657</v>
       </c>
       <c r="R64" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S64" s="54" t="s">
+      <c r="S64" s="50" t="s">
         <v>113</v>
       </c>
-      <c r="AK64" s="55"/>
+      <c r="AK64" s="51"/>
       <c r="AL64" s="2"/>
       <c r="AM64" s="3"/>
       <c r="AN64" s="3"/>
@@ -3058,16 +3038,16 @@
       <c r="O65" s="46" t="n">
         <v>0.001764</v>
       </c>
-      <c r="P65" s="56" t="n">
+      <c r="P65" s="52" t="n">
         <v>99873.4773901073</v>
       </c>
-      <c r="Q65" s="57" t="n">
+      <c r="Q65" s="53" t="n">
         <v>318.01399715178</v>
       </c>
       <c r="R65" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S65" s="54" t="s">
+      <c r="S65" s="50" t="s">
         <v>130</v>
       </c>
       <c r="AL65" s="2"/>
@@ -3119,19 +3099,19 @@
       <c r="O66" s="46" t="n">
         <v>0.000511</v>
       </c>
-      <c r="P66" s="56" t="n">
+      <c r="P66" s="52" t="n">
         <v>85045.2462252718</v>
       </c>
-      <c r="Q66" s="57" t="n">
+      <c r="Q66" s="53" t="n">
         <v>292.351904129881</v>
       </c>
       <c r="R66" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S66" s="54" t="s">
+      <c r="S66" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="AK66" s="55"/>
+      <c r="AK66" s="51"/>
       <c r="AL66" s="2"/>
       <c r="AM66" s="3"/>
       <c r="AN66" s="3"/>
@@ -3181,19 +3161,19 @@
       <c r="O67" s="46" t="n">
         <v>0.000516</v>
       </c>
-      <c r="P67" s="56" t="n">
+      <c r="P67" s="52" t="n">
         <v>98251.0314876961</v>
       </c>
-      <c r="Q67" s="57" t="n">
+      <c r="Q67" s="53" t="n">
         <v>315.666474205925</v>
       </c>
       <c r="R67" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S67" s="54" t="s">
+      <c r="S67" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="AK67" s="55"/>
+      <c r="AK67" s="51"/>
       <c r="AL67" s="2"/>
       <c r="AM67" s="3"/>
       <c r="AN67" s="3"/>
@@ -3243,16 +3223,16 @@
       <c r="O68" s="46" t="n">
         <v>0.001569</v>
       </c>
-      <c r="P68" s="56" t="n">
+      <c r="P68" s="52" t="n">
         <v>82992.5578598319</v>
       </c>
-      <c r="Q68" s="57" t="n">
+      <c r="Q68" s="53" t="n">
         <v>289.835162889762</v>
       </c>
       <c r="R68" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S68" s="54" t="s">
+      <c r="S68" s="50" t="s">
         <v>130</v>
       </c>
       <c r="AL68" s="2"/>
@@ -3304,16 +3284,16 @@
       <c r="O69" s="46" t="n">
         <v>0.001603</v>
       </c>
-      <c r="P69" s="56" t="n">
+      <c r="P69" s="52" t="n">
         <v>55605.7041292573</v>
       </c>
-      <c r="Q69" s="57" t="n">
+      <c r="Q69" s="53" t="n">
         <v>236.980358232231</v>
       </c>
       <c r="R69" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S69" s="54" t="s">
+      <c r="S69" s="50" t="s">
         <v>130</v>
       </c>
       <c r="AL69" s="2"/>
@@ -3365,16 +3345,16 @@
       <c r="O70" s="46" t="n">
         <v>0.001532</v>
       </c>
-      <c r="P70" s="56" t="n">
+      <c r="P70" s="52" t="n">
         <v>57590.915602123</v>
       </c>
-      <c r="Q70" s="57" t="n">
+      <c r="Q70" s="53" t="n">
         <v>240.865244134391</v>
       </c>
       <c r="R70" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S70" s="54" t="s">
+      <c r="S70" s="50" t="s">
         <v>130</v>
       </c>
       <c r="AL70" s="2"/>
@@ -3426,19 +3406,19 @@
       <c r="O71" s="46" t="n">
         <v>0.000164</v>
       </c>
-      <c r="P71" s="56" t="n">
+      <c r="P71" s="52" t="n">
         <v>47402.2973352247</v>
       </c>
-      <c r="Q71" s="57" t="n">
+      <c r="Q71" s="53" t="n">
         <v>226.618540463308</v>
       </c>
       <c r="R71" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S71" s="54" t="s">
+      <c r="S71" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="AK71" s="55"/>
+      <c r="AK71" s="51"/>
       <c r="AL71" s="2"/>
       <c r="AM71" s="3"/>
       <c r="AN71" s="3"/>
@@ -3488,19 +3468,19 @@
       <c r="O72" s="46" t="n">
         <v>0.000213</v>
       </c>
-      <c r="P72" s="56" t="n">
+      <c r="P72" s="52" t="n">
         <v>31385.3739775756</v>
       </c>
-      <c r="Q72" s="57" t="n">
+      <c r="Q72" s="53" t="n">
         <v>179.005904347796</v>
       </c>
       <c r="R72" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S72" s="54" t="s">
+      <c r="S72" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="AK72" s="55"/>
+      <c r="AK72" s="51"/>
       <c r="AL72" s="2"/>
       <c r="AM72" s="3"/>
       <c r="AN72" s="3"/>
@@ -3550,19 +3530,19 @@
       <c r="O73" s="46" t="n">
         <v>0.001494</v>
       </c>
-      <c r="P73" s="56" t="n">
+      <c r="P73" s="52" t="n">
         <v>35492.6155876485</v>
       </c>
-      <c r="Q73" s="57" t="n">
+      <c r="Q73" s="53" t="n">
         <v>193.935510485773</v>
       </c>
       <c r="R73" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S73" s="54" t="s">
+      <c r="S73" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="AK73" s="55"/>
+      <c r="AK73" s="51"/>
       <c r="AL73" s="2"/>
       <c r="AM73" s="3"/>
       <c r="AN73" s="3"/>
@@ -3612,16 +3592,16 @@
       <c r="O74" s="46" t="n">
         <v>0.001502</v>
       </c>
-      <c r="P74" s="56" t="n">
+      <c r="P74" s="52" t="n">
         <v>384707.454376199</v>
       </c>
-      <c r="Q74" s="57" t="n">
+      <c r="Q74" s="53" t="n">
         <v>625.587607003867</v>
       </c>
       <c r="R74" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="S74" s="54" t="s">
+      <c r="S74" s="50" t="s">
         <v>113</v>
       </c>
       <c r="AL74" s="2"/>
@@ -3630,59 +3610,59 @@
       <c r="AO74" s="2"/>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="58"/>
-      <c r="B75" s="59" t="s">
+      <c r="A75" s="54"/>
+      <c r="B75" s="55" t="s">
         <v>167</v>
       </c>
-      <c r="C75" s="60" t="n">
+      <c r="C75" s="56" t="n">
         <v>791970</v>
       </c>
-      <c r="D75" s="60" t="n">
+      <c r="D75" s="56" t="n">
         <v>102</v>
       </c>
-      <c r="E75" s="59" t="s">
+      <c r="E75" s="55" t="s">
         <v>168</v>
       </c>
-      <c r="F75" s="60" t="n">
+      <c r="F75" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="G75" s="59" t="n">
+      <c r="G75" s="55" t="n">
         <v>50</v>
       </c>
-      <c r="H75" s="59" t="s">
+      <c r="H75" s="55" t="s">
         <v>109</v>
       </c>
-      <c r="I75" s="59" t="s">
+      <c r="I75" s="55" t="s">
         <v>169</v>
       </c>
-      <c r="J75" s="59" t="s">
+      <c r="J75" s="55" t="s">
         <v>170</v>
       </c>
-      <c r="K75" s="59" t="s">
+      <c r="K75" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="L75" s="59" t="s">
+      <c r="L75" s="55" t="s">
         <v>112</v>
       </c>
-      <c r="M75" s="59" t="n">
+      <c r="M75" s="55" t="n">
         <v>190308.826168728</v>
       </c>
-      <c r="N75" s="59" t="n">
+      <c r="N75" s="55" t="n">
         <v>438.281965184008</v>
       </c>
-      <c r="O75" s="59" t="n">
+      <c r="O75" s="55" t="n">
         <v>0.000321</v>
       </c>
-      <c r="P75" s="61" t="n">
+      <c r="P75" s="57" t="n">
         <v>190247.825198091</v>
       </c>
-      <c r="Q75" s="62" t="n">
+      <c r="Q75" s="58" t="n">
         <v>438.211072069943</v>
       </c>
-      <c r="R75" s="63" t="n">
+      <c r="R75" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="S75" s="64" t="s">
+      <c r="S75" s="60" t="s">
         <v>113</v>
       </c>
       <c r="AL75" s="2"/>
@@ -3693,7 +3673,7 @@
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="R76" s="3"/>
       <c r="S76" s="2"/>
-      <c r="AK76" s="55"/>
+      <c r="AK76" s="51"/>
       <c r="AL76" s="2"/>
       <c r="AM76" s="3"/>
       <c r="AN76" s="3"/>
@@ -3708,20 +3688,20 @@
       <c r="AO77" s="2"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O78" s="55"/>
+      <c r="O78" s="51"/>
       <c r="R78" s="3"/>
       <c r="S78" s="2"/>
-      <c r="AK78" s="55"/>
+      <c r="AK78" s="51"/>
       <c r="AL78" s="2"/>
       <c r="AM78" s="3"/>
       <c r="AN78" s="3"/>
       <c r="AO78" s="2"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O79" s="55"/>
+      <c r="O79" s="51"/>
       <c r="R79" s="3"/>
       <c r="S79" s="2"/>
-      <c r="AK79" s="55"/>
+      <c r="AK79" s="51"/>
       <c r="AL79" s="2"/>
       <c r="AM79" s="3"/>
       <c r="AN79" s="3"/>
@@ -3736,7 +3716,7 @@
       <c r="AO80" s="2"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O81" s="55"/>
+      <c r="O81" s="51"/>
       <c r="R81" s="3"/>
       <c r="S81" s="2"/>
       <c r="AL81" s="2"/>
@@ -3745,7 +3725,7 @@
       <c r="AO81" s="2"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O82" s="55"/>
+      <c r="O82" s="51"/>
       <c r="R82" s="3"/>
       <c r="S82" s="2"/>
       <c r="AL82" s="2"/>
@@ -3756,7 +3736,7 @@
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="R83" s="3"/>
       <c r="S83" s="2"/>
-      <c r="AK83" s="55"/>
+      <c r="AK83" s="51"/>
       <c r="AL83" s="2"/>
       <c r="AM83" s="3"/>
       <c r="AN83" s="3"/>
@@ -3779,7 +3759,7 @@
       <c r="AO85" s="2"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O86" s="55"/>
+      <c r="O86" s="51"/>
       <c r="R86" s="3"/>
       <c r="S86" s="2"/>
       <c r="AL86" s="2"/>
@@ -3978,7 +3958,7 @@
       <c r="R130" s="3"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B131" s="65"/>
+      <c r="B131" s="61"/>
       <c r="R131" s="3"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4301,7 +4281,7 @@
       <c r="R234" s="3"/>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="L235" s="66"/>
+      <c r="L235" s="62"/>
       <c r="R235" s="3"/>
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4373,7 +4353,7 @@
       <c r="R257" s="3"/>
     </row>
     <row r="258" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O258" s="55"/>
+      <c r="O258" s="51"/>
       <c r="R258" s="3"/>
     </row>
     <row r="259" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4574,7 +4554,7 @@
       <c r="R321" s="3"/>
     </row>
     <row r="322" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O322" s="55"/>
+      <c r="O322" s="51"/>
       <c r="R322" s="3"/>
     </row>
     <row r="323" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4641,11 +4621,11 @@
       <c r="R343" s="3"/>
     </row>
     <row r="344" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K344" s="67"/>
+      <c r="K344" s="63"/>
       <c r="R344" s="3"/>
     </row>
     <row r="345" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K345" s="67"/>
+      <c r="K345" s="63"/>
       <c r="R345" s="3"/>
     </row>
     <row r="346" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4767,7 +4747,7 @@
       <c r="R393" s="3"/>
     </row>
     <row r="394" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O394" s="55"/>
+      <c r="O394" s="51"/>
       <c r="R394" s="3"/>
     </row>
     <row r="395" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4780,11 +4760,11 @@
       <c r="R397" s="3"/>
     </row>
     <row r="398" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O398" s="55"/>
+      <c r="O398" s="51"/>
       <c r="R398" s="3"/>
     </row>
     <row r="399" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O399" s="55"/>
+      <c r="O399" s="51"/>
       <c r="R399" s="3"/>
     </row>
     <row r="400" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4800,14 +4780,14 @@
       <c r="R403" s="3"/>
     </row>
     <row r="404" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O404" s="55"/>
+      <c r="O404" s="51"/>
       <c r="R404" s="3"/>
     </row>
     <row r="405" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R405" s="3"/>
     </row>
     <row r="406" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O406" s="55"/>
+      <c r="O406" s="51"/>
       <c r="R406" s="3"/>
     </row>
     <row r="407" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4963,7 +4943,7 @@
       <c r="R456" s="3"/>
     </row>
     <row r="457" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O457" s="55"/>
+      <c r="O457" s="51"/>
       <c r="R457" s="3"/>
     </row>
     <row r="458" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5111,14 +5091,14 @@
     </row>
     <row r="505" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R505" s="3"/>
-      <c r="AE505" s="67"/>
+      <c r="AE505" s="63"/>
       <c r="AJ505" s="2"/>
       <c r="AK505" s="3"/>
       <c r="AL505" s="3"/>
     </row>
     <row r="506" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R506" s="3"/>
-      <c r="AE506" s="67"/>
+      <c r="AE506" s="63"/>
       <c r="AJ506" s="2"/>
       <c r="AK506" s="3"/>
       <c r="AL506" s="3"/>
@@ -5151,7 +5131,7 @@
     <row r="511" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="M511" s="7"/>
       <c r="R511" s="3"/>
-      <c r="AF511" s="68"/>
+      <c r="AF511" s="64"/>
       <c r="AJ511" s="2"/>
       <c r="AK511" s="3"/>
       <c r="AL511" s="3"/>
@@ -5304,7 +5284,7 @@
       <c r="AL536" s="3"/>
     </row>
     <row r="537" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C537" s="69"/>
+      <c r="C537" s="65"/>
       <c r="R537" s="3"/>
       <c r="AJ537" s="2"/>
       <c r="AK537" s="3"/>
@@ -5324,7 +5304,7 @@
     </row>
     <row r="540" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R540" s="3"/>
-      <c r="AI540" s="55"/>
+      <c r="AI540" s="51"/>
       <c r="AJ540" s="2"/>
       <c r="AK540" s="3"/>
       <c r="AL540" s="3"/>
@@ -5343,21 +5323,21 @@
     </row>
     <row r="543" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R543" s="3"/>
-      <c r="AI543" s="55"/>
+      <c r="AI543" s="51"/>
       <c r="AJ543" s="2"/>
       <c r="AK543" s="3"/>
       <c r="AL543" s="3"/>
     </row>
     <row r="544" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R544" s="3"/>
-      <c r="AI544" s="55"/>
+      <c r="AI544" s="51"/>
       <c r="AJ544" s="2"/>
       <c r="AK544" s="3"/>
       <c r="AL544" s="3"/>
     </row>
     <row r="545" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R545" s="3"/>
-      <c r="AI545" s="55"/>
+      <c r="AI545" s="51"/>
       <c r="AJ545" s="2"/>
       <c r="AK545" s="3"/>
       <c r="AL545" s="3"/>
@@ -5390,7 +5370,7 @@
     </row>
     <row r="550" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R550" s="3"/>
-      <c r="AI550" s="55"/>
+      <c r="AI550" s="51"/>
       <c r="AJ550" s="2"/>
       <c r="AK550" s="3"/>
       <c r="AL550" s="3"/>
@@ -5403,7 +5383,7 @@
     </row>
     <row r="552" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R552" s="3"/>
-      <c r="AI552" s="55"/>
+      <c r="AI552" s="51"/>
       <c r="AJ552" s="2"/>
       <c r="AK552" s="3"/>
       <c r="AL552" s="3"/>
@@ -5416,7 +5396,7 @@
     </row>
     <row r="554" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R554" s="3"/>
-      <c r="AI554" s="55"/>
+      <c r="AI554" s="51"/>
       <c r="AJ554" s="2"/>
       <c r="AK554" s="3"/>
       <c r="AL554" s="3"/>
@@ -5435,21 +5415,21 @@
     </row>
     <row r="557" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R557" s="3"/>
-      <c r="AI557" s="55"/>
+      <c r="AI557" s="51"/>
       <c r="AJ557" s="2"/>
       <c r="AK557" s="3"/>
       <c r="AL557" s="3"/>
     </row>
     <row r="558" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R558" s="3"/>
-      <c r="AI558" s="55"/>
+      <c r="AI558" s="51"/>
       <c r="AJ558" s="2"/>
       <c r="AK558" s="3"/>
       <c r="AL558" s="3"/>
     </row>
     <row r="559" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R559" s="3"/>
-      <c r="AI559" s="55"/>
+      <c r="AI559" s="51"/>
       <c r="AJ559" s="2"/>
       <c r="AK559" s="3"/>
       <c r="AL559" s="3"/>
@@ -5480,7 +5460,7 @@
     </row>
     <row r="564" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R564" s="3"/>
-      <c r="AI564" s="55"/>
+      <c r="AI564" s="51"/>
       <c r="AJ564" s="2"/>
       <c r="AK564" s="3"/>
       <c r="AL564" s="3"/>
@@ -5493,7 +5473,7 @@
     </row>
     <row r="566" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R566" s="3"/>
-      <c r="AI566" s="55"/>
+      <c r="AI566" s="51"/>
       <c r="AJ566" s="2"/>
       <c r="AK566" s="3"/>
       <c r="AL566" s="3"/>
@@ -5505,7 +5485,7 @@
       <c r="AL567" s="3"/>
     </row>
     <row r="568" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O568" s="55"/>
+      <c r="O568" s="51"/>
       <c r="R568" s="3"/>
       <c r="AJ568" s="2"/>
       <c r="AK568" s="3"/>
@@ -5549,7 +5529,7 @@
     </row>
     <row r="575" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R575" s="3"/>
-      <c r="T575" s="69"/>
+      <c r="T575" s="65"/>
       <c r="AJ575" s="2"/>
       <c r="AK575" s="3"/>
       <c r="AL575" s="3"/>
@@ -5645,17 +5625,17 @@
       <c r="R598" s="3"/>
     </row>
     <row r="599" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K599" s="67"/>
+      <c r="K599" s="63"/>
       <c r="R599" s="3"/>
-      <c r="AF599" s="67"/>
+      <c r="AF599" s="63"/>
       <c r="AK599" s="2"/>
       <c r="AL599" s="3"/>
       <c r="AM599" s="3"/>
     </row>
     <row r="600" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K600" s="67"/>
+      <c r="K600" s="63"/>
       <c r="R600" s="3"/>
-      <c r="AF600" s="67"/>
+      <c r="AF600" s="63"/>
       <c r="AK600" s="2"/>
       <c r="AL600" s="3"/>
       <c r="AM600" s="3"/>
@@ -5685,9 +5665,9 @@
       <c r="AM604" s="3"/>
     </row>
     <row r="605" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L605" s="68"/>
+      <c r="L605" s="64"/>
       <c r="R605" s="3"/>
-      <c r="AG605" s="68"/>
+      <c r="AG605" s="64"/>
       <c r="AK605" s="2"/>
       <c r="AL605" s="3"/>
       <c r="AM605" s="3"/>
@@ -5856,7 +5836,7 @@
     </row>
     <row r="634" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R634" s="3"/>
-      <c r="AJ634" s="55"/>
+      <c r="AJ634" s="51"/>
       <c r="AK634" s="2"/>
       <c r="AL634" s="3"/>
       <c r="AM634" s="3"/>
@@ -5875,21 +5855,21 @@
     </row>
     <row r="637" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R637" s="3"/>
-      <c r="AJ637" s="55"/>
+      <c r="AJ637" s="51"/>
       <c r="AK637" s="2"/>
       <c r="AL637" s="3"/>
       <c r="AM637" s="3"/>
     </row>
     <row r="638" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R638" s="3"/>
-      <c r="AJ638" s="55"/>
+      <c r="AJ638" s="51"/>
       <c r="AK638" s="2"/>
       <c r="AL638" s="3"/>
       <c r="AM638" s="3"/>
     </row>
     <row r="639" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R639" s="3"/>
-      <c r="AJ639" s="55"/>
+      <c r="AJ639" s="51"/>
       <c r="AK639" s="2"/>
       <c r="AL639" s="3"/>
       <c r="AM639" s="3"/>
@@ -5920,7 +5900,7 @@
     </row>
     <row r="644" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R644" s="3"/>
-      <c r="AJ644" s="55"/>
+      <c r="AJ644" s="51"/>
       <c r="AK644" s="2"/>
       <c r="AL644" s="3"/>
       <c r="AM644" s="3"/>
@@ -5933,7 +5913,7 @@
     </row>
     <row r="646" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R646" s="3"/>
-      <c r="AJ646" s="55"/>
+      <c r="AJ646" s="51"/>
       <c r="AK646" s="2"/>
       <c r="AL646" s="3"/>
       <c r="AM646" s="3"/>
@@ -5946,7 +5926,7 @@
     </row>
     <row r="648" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R648" s="3"/>
-      <c r="AJ648" s="55"/>
+      <c r="AJ648" s="51"/>
       <c r="AK648" s="2"/>
       <c r="AL648" s="3"/>
       <c r="AM648" s="3"/>
@@ -5958,7 +5938,7 @@
       <c r="AM649" s="3"/>
     </row>
     <row r="650" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O650" s="55"/>
+      <c r="O650" s="51"/>
       <c r="R650" s="3"/>
       <c r="AK650" s="2"/>
       <c r="AL650" s="3"/>
@@ -5966,35 +5946,35 @@
     </row>
     <row r="651" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R651" s="3"/>
-      <c r="AJ651" s="55"/>
+      <c r="AJ651" s="51"/>
       <c r="AK651" s="2"/>
       <c r="AL651" s="3"/>
       <c r="AM651" s="3"/>
     </row>
     <row r="652" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R652" s="3"/>
-      <c r="AJ652" s="55"/>
+      <c r="AJ652" s="51"/>
       <c r="AK652" s="2"/>
       <c r="AL652" s="3"/>
       <c r="AM652" s="3"/>
     </row>
     <row r="653" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O653" s="55"/>
+      <c r="O653" s="51"/>
       <c r="R653" s="3"/>
-      <c r="AJ653" s="55"/>
+      <c r="AJ653" s="51"/>
       <c r="AK653" s="2"/>
       <c r="AL653" s="3"/>
       <c r="AM653" s="3"/>
     </row>
     <row r="654" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O654" s="55"/>
+      <c r="O654" s="51"/>
       <c r="R654" s="3"/>
       <c r="AK654" s="2"/>
       <c r="AL654" s="3"/>
       <c r="AM654" s="3"/>
     </row>
     <row r="655" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O655" s="55"/>
+      <c r="O655" s="51"/>
       <c r="R655" s="3"/>
       <c r="AK655" s="2"/>
       <c r="AL655" s="3"/>
@@ -6014,7 +5994,7 @@
     </row>
     <row r="658" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R658" s="3"/>
-      <c r="AJ658" s="55"/>
+      <c r="AJ658" s="51"/>
       <c r="AK658" s="2"/>
       <c r="AL658" s="3"/>
       <c r="AM658" s="3"/>
@@ -6026,9 +6006,9 @@
       <c r="AM659" s="3"/>
     </row>
     <row r="660" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O660" s="55"/>
+      <c r="O660" s="51"/>
       <c r="R660" s="3"/>
-      <c r="AJ660" s="55"/>
+      <c r="AJ660" s="51"/>
       <c r="AK660" s="2"/>
       <c r="AL660" s="3"/>
       <c r="AM660" s="3"/>
@@ -6040,7 +6020,7 @@
       <c r="AM661" s="3"/>
     </row>
     <row r="662" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O662" s="55"/>
+      <c r="O662" s="51"/>
       <c r="R662" s="3"/>
       <c r="AK662" s="2"/>
       <c r="AL662" s="3"/>
@@ -6150,7 +6130,7 @@
       <c r="R681" s="3"/>
     </row>
     <row r="682" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C682" s="70"/>
+      <c r="C682" s="66"/>
       <c r="R682" s="3"/>
     </row>
     <row r="683" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6398,7 +6378,7 @@
       <c r="R762" s="3"/>
     </row>
     <row r="763" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D763" s="70"/>
+      <c r="D763" s="66"/>
       <c r="R763" s="3"/>
     </row>
     <row r="764" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6509,7 +6489,7 @@
       <c r="R798" s="3"/>
     </row>
     <row r="799" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D799" s="70"/>
+      <c r="D799" s="66"/>
       <c r="R799" s="3"/>
     </row>
     <row r="800" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6650,12 +6630,12 @@
       <c r="R844" s="3"/>
     </row>
     <row r="845" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C845" s="70"/>
-      <c r="K845" s="67"/>
+      <c r="C845" s="66"/>
+      <c r="K845" s="63"/>
       <c r="R845" s="3"/>
     </row>
     <row r="846" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K846" s="67"/>
+      <c r="K846" s="63"/>
       <c r="R846" s="3"/>
     </row>
     <row r="847" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6781,7 +6761,7 @@
     </row>
     <row r="880" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R880" s="3"/>
-      <c r="AK880" s="55"/>
+      <c r="AK880" s="51"/>
       <c r="AL880" s="2"/>
       <c r="AM880" s="3"/>
       <c r="AN880" s="3"/>
@@ -6806,14 +6786,14 @@
     </row>
     <row r="884" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R884" s="3"/>
-      <c r="AK884" s="55"/>
+      <c r="AK884" s="51"/>
       <c r="AL884" s="2"/>
       <c r="AM884" s="3"/>
       <c r="AN884" s="3"/>
     </row>
     <row r="885" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R885" s="3"/>
-      <c r="AK885" s="55"/>
+      <c r="AK885" s="51"/>
       <c r="AL885" s="2"/>
       <c r="AM885" s="3"/>
       <c r="AN885" s="3"/>
@@ -6856,7 +6836,7 @@
     </row>
     <row r="892" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R892" s="3"/>
-      <c r="AK892" s="55"/>
+      <c r="AK892" s="51"/>
       <c r="AL892" s="2"/>
       <c r="AM892" s="3"/>
       <c r="AN892" s="3"/>
@@ -6869,7 +6849,7 @@
     </row>
     <row r="894" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R894" s="3"/>
-      <c r="AK894" s="55"/>
+      <c r="AK894" s="51"/>
       <c r="AL894" s="2"/>
       <c r="AM894" s="3"/>
       <c r="AN894" s="3"/>
@@ -6881,7 +6861,7 @@
       <c r="AN895" s="3"/>
     </row>
     <row r="896" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O896" s="55"/>
+      <c r="O896" s="51"/>
       <c r="R896" s="3"/>
       <c r="AL896" s="2"/>
       <c r="AM896" s="3"/>
@@ -6895,27 +6875,27 @@
     </row>
     <row r="898" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R898" s="3"/>
-      <c r="AK898" s="55"/>
+      <c r="AK898" s="51"/>
       <c r="AL898" s="2"/>
       <c r="AM898" s="3"/>
       <c r="AN898" s="3"/>
     </row>
     <row r="899" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R899" s="3"/>
-      <c r="AK899" s="55"/>
+      <c r="AK899" s="51"/>
       <c r="AL899" s="2"/>
       <c r="AM899" s="3"/>
       <c r="AN899" s="3"/>
     </row>
     <row r="900" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O900" s="55"/>
+      <c r="O900" s="51"/>
       <c r="R900" s="3"/>
       <c r="AL900" s="2"/>
       <c r="AM900" s="3"/>
       <c r="AN900" s="3"/>
     </row>
     <row r="901" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O901" s="55"/>
+      <c r="O901" s="51"/>
       <c r="R901" s="3"/>
       <c r="AL901" s="2"/>
       <c r="AM901" s="3"/>
@@ -6947,7 +6927,7 @@
     </row>
     <row r="906" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R906" s="3"/>
-      <c r="AK906" s="55"/>
+      <c r="AK906" s="51"/>
       <c r="AL906" s="2"/>
       <c r="AM906" s="3"/>
       <c r="AN906" s="3"/>
@@ -6959,7 +6939,7 @@
       <c r="AN907" s="3"/>
     </row>
     <row r="908" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O908" s="55"/>
+      <c r="O908" s="51"/>
       <c r="R908" s="3"/>
       <c r="AL908" s="2"/>
       <c r="AM908" s="3"/>
@@ -7462,11 +7442,11 @@
     </row>
     <row r="1057" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R1057" s="3"/>
-      <c r="T1057" s="71"/>
+      <c r="T1057" s="67"/>
     </row>
     <row r="1058" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R1058" s="3"/>
-      <c r="T1058" s="72"/>
+      <c r="T1058" s="11"/>
     </row>
     <row r="1059" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="R1059" s="3"/>
@@ -7481,7 +7461,7 @@
       <c r="R1062" s="3"/>
     </row>
     <row r="1063" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O1063" s="55"/>
+      <c r="O1063" s="51"/>
       <c r="R1063" s="3"/>
     </row>
     <row r="1064" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>